<commit_message>
47차: Stage3 복귀 HUD 정리 및 Stage4 MFC 표시 안정화
CookingGroup에서 EncounterGroup으로 복귀할 때 인벤토리 HUD가 대화 패널을 가리지 않도록 강제 닫기 흐름을 추가했다.

인벤토리 자동 오픈 큐와 복귀 타이밍이 충돌하지 않도록 즉시/지연 재시도 방식으로 안정화했다.

CookingGroup의 임무 완수 안내가 더 잘 보이도록 검은 배경과 흰 글씨 대비를 강화했다.

4th_Road_to_Stage4 진입 시 MFC가 보이지 않던 문제를 수정했다.

깨진 MFC 스프라이트/애니메이터 참조를 정상 리소스로 복구하고, RoadGroup에서 유효한 MFC 오브젝트를 우선 선택하도록 보강했다.

Unity batchmode로 Stage4 MFC가 맵 안, 카메라 안, 정상 스프라이트 상태로 표시되는지 검증했다.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OO_Stage4CueSheet.xlsx
+++ b/JsonConverter/ExcelFiles/OO_Stage4CueSheet.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD4"/>
+  <dimension ref="A1:AF4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -508,120 +508,130 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Road 임무 데이터 ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Road 임무 fallback 문장</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>거북이 역할 ID</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>토끼 역할 ID</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>잠든 토끼 역할 ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>모란 역할 ID</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>그루터기 역할 ID</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>전환 그루터기 역할 ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>정지 포인트 A 역할 ID</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>거북이 시작 대사 목록</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>거북이 완료 대사 목록</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>토끼 첫 대사 ID</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>토끼 정지점 대사 ID</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>당근전 보유 후 토끼 대사 목록</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>토끼 말풍선 ID 목록</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>잠든 토끼 말풍선 ID</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>스테이지4 퀘스트 ID</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>당근 재료 ID</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>떡 음식 ID</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>당근전분 음식 ID</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>당근전 음식 ID</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Stage4 BGM 경로</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>최종 튜토리얼 나레이션 ID</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>상호작용 거리</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>토끼 달리기 속도</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>토끼 강제 도착 시간</t>
         </is>
@@ -765,15 +775,25 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
           <t>float</t>
         </is>
       </c>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="AD2" s="2" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -812,120 +832,130 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>RoadMissionDataId</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>RoadMissionFallbackText</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
           <t>TurtleRoleId</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>RabbitRoleId</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>SleepingRabbitRoleId</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>MoranRoleId</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>StumpRoleId</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Stump2RoleId</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>StopPointARoleId</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>TurtleDialogueIdList</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>TurtleClearDialogueIdList</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>RabbitIntroDialogueId</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>RabbitStopDialogueId</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>RabbitCarrotCakeDialogueIdList</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>RabbitSpeechBubbleIdList</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="V3" s="3" t="inlineStr">
         <is>
           <t>RabbitSleepingBubbleId</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="W3" s="3" t="inlineStr">
         <is>
           <t>StageQuestId</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="X3" s="3" t="inlineStr">
         <is>
           <t>CarrotIngredientId</t>
         </is>
       </c>
-      <c r="W3" s="3" t="inlineStr">
+      <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>KoreanCakeItemId</t>
         </is>
       </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="Z3" s="3" t="inlineStr">
         <is>
           <t>CarrotStarchItemId</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="AA3" s="3" t="inlineStr">
         <is>
           <t>CarrotCakeItemId</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="AB3" s="3" t="inlineStr">
         <is>
           <t>Stage4BGMPath</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AC3" s="3" t="inlineStr">
         <is>
           <t>NextTutorialNarrationId</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
+      <c r="AD3" s="3" t="inlineStr">
         <is>
           <t>InteractionDistance</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="inlineStr">
+      <c r="AE3" s="3" t="inlineStr">
         <is>
           <t>RabbitRunSpeed</t>
         </is>
       </c>
-      <c r="AD3" s="3" t="inlineStr">
+      <c r="AF3" s="3" t="inlineStr">
         <is>
           <t>RabbitReachTimeoutSeconds</t>
         </is>
@@ -964,116 +994,126 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Stage4_Road_Quest_01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>북쪽 농경지대로 가세요.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>Turtle</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Rabbit_isSleeping</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Moran</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Stump</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Stump2</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>StopPoint_A</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>character_Turtle_01|character_Turtle_02</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>character_Turtle_03|character_Turtle_04</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>character_Rabbit_01</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>character_Rabbit_02</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>character_Rabbit_03|character_Rabbit_04</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>character_Rabbit_01|character_Rabbit_02|character_Rabbit_03|character_Rabbit_04|character_Rabbit_05</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>character_Rabbit_06</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Stage4__Quest_01</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Ing_Carrot_01</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>OO_KoreanCake_1</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>OO_CarrotStarch_1</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>OO_CarrotCake_1</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>Audio/BGM/Stage4_BGM</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>narration_tutorial_15</t>
         </is>
       </c>
-      <c r="AB4" t="n">
+      <c r="AD4" t="n">
         <v>95</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AE4" t="n">
         <v>480</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AF4" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>